<commit_message>
feat(report): refresh V817 sections 6-9 (Jan2026+/2025/2024/2021-23) on new ticks
</commit_message>
<xml_diff>
--- a/reports/V817_2021_2023.xlsx
+++ b/reports/V817_2021_2023.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Daily Breakdown" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Per-Entry Detail" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Weekly Breakdown" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Daily Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Per-Entry Detail" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -679,7 +680,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-06-29 10:02:00</t>
+          <t>2026-06-29 19:07:00</t>
         </is>
       </c>
     </row>
@@ -1005,6 +1006,96 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Month-Week</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Signals</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Wins</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Losses</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>No-fills</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Win rate</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Trading P&amp;L</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Bonus</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Closed lots</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Net P&amp;L</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Equity EoW</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1106,7 +1197,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>